<commit_message>
Update import logic and UI based on feedback
</commit_message>
<xml_diff>
--- a/public/format_import_siswa.xlsx
+++ b/public/format_import_siswa.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>nis</t>
   </si>
@@ -31,12 +31,6 @@
     <t>birth_date</t>
   </si>
   <si>
-    <t>class_name</t>
-  </si>
-  <si>
-    <t>major_code</t>
-  </si>
-  <si>
     <t>parent_name</t>
   </si>
   <si>
@@ -46,9 +40,6 @@
     <t>phone</t>
   </si>
   <si>
-    <t>graduation_status</t>
-  </si>
-  <si>
     <t>1001</t>
   </si>
   <si>
@@ -67,12 +58,6 @@
     <t>2005-01-01</t>
   </si>
   <si>
-    <t>XII RPL 1</t>
-  </si>
-  <si>
-    <t>RPL</t>
-  </si>
-  <si>
     <t>Santoso</t>
   </si>
   <si>
@@ -80,9 +65,6 @@
   </si>
   <si>
     <t>08123456789</t>
-  </si>
-  <si>
-    <t>LULUS</t>
   </si>
 </sst>
 </file>
@@ -459,20 +441,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="15" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="25" customWidth="1"/>
-    <col min="10" max="10" width="30" customWidth="1"/>
-    <col min="11" max="11" width="15" customWidth="1"/>
-    <col min="12" max="12" width="20" customWidth="1"/>
+    <col min="5" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="25" customWidth="1"/>
+    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -500,52 +481,34 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="B2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="C2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="D2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" t="s">
+      <c r="E2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" t="s">
+      <c r="F2" t="s">
         <v>14</v>
       </c>
-      <c r="D2" t="s">
+      <c r="G2" t="s">
         <v>15</v>
       </c>
-      <c r="E2" t="s">
+      <c r="H2" t="s">
         <v>16</v>
       </c>
-      <c r="F2" t="s">
+      <c r="I2" t="s">
         <v>17</v>
-      </c>
-      <c r="G2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L2" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>